<commit_message>
Daily follower scan: 2026-09-14
</commit_message>
<xml_diff>
--- a/daily_report.xlsx
+++ b/daily_report.xlsx
@@ -450,16 +450,16 @@
         </is>
       </c>
       <c r="B2" t="n">
+        <v>409673</v>
+      </c>
+      <c r="C2" t="n">
         <v>409540</v>
       </c>
-      <c r="C2" t="n">
-        <v>409401</v>
-      </c>
       <c r="D2" t="n">
-        <v>139</v>
+        <v>133</v>
       </c>
       <c r="E2" t="n">
-        <v>0.034</v>
+        <v>0.0325</v>
       </c>
     </row>
     <row r="3">
@@ -469,16 +469,16 @@
         </is>
       </c>
       <c r="B3" t="n">
+        <v>2496796</v>
+      </c>
+      <c r="C3" t="n">
         <v>2496824</v>
       </c>
-      <c r="C3" t="n">
-        <v>2496794</v>
-      </c>
       <c r="D3" t="n">
-        <v>30</v>
+        <v>-28</v>
       </c>
       <c r="E3" t="n">
-        <v>0.0012</v>
+        <v>-0.0011</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily follower scan: 2026-09-15
</commit_message>
<xml_diff>
--- a/daily_report.xlsx
+++ b/daily_report.xlsx
@@ -450,16 +450,16 @@
         </is>
       </c>
       <c r="B2" t="n">
+        <v>409739</v>
+      </c>
+      <c r="C2" t="n">
         <v>409673</v>
       </c>
-      <c r="C2" t="n">
-        <v>409540</v>
-      </c>
       <c r="D2" t="n">
-        <v>133</v>
+        <v>66</v>
       </c>
       <c r="E2" t="n">
-        <v>0.0325</v>
+        <v>0.0161</v>
       </c>
     </row>
     <row r="3">
@@ -469,16 +469,16 @@
         </is>
       </c>
       <c r="B3" t="n">
+        <v>2496757</v>
+      </c>
+      <c r="C3" t="n">
         <v>2496796</v>
       </c>
-      <c r="C3" t="n">
-        <v>2496824</v>
-      </c>
       <c r="D3" t="n">
-        <v>-28</v>
+        <v>-39</v>
       </c>
       <c r="E3" t="n">
-        <v>-0.0011</v>
+        <v>-0.0016</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily follower scan: 2026-09-16
</commit_message>
<xml_diff>
--- a/daily_report.xlsx
+++ b/daily_report.xlsx
@@ -446,39 +446,39 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>myxl</t>
+          <t>telkomsel</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>409739</v>
+        <v>2496649</v>
       </c>
       <c r="C2" t="n">
-        <v>409673</v>
+        <v>2496757</v>
       </c>
       <c r="D2" t="n">
-        <v>66</v>
+        <v>-108</v>
       </c>
       <c r="E2" t="n">
-        <v>0.0161</v>
+        <v>-0.0043</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>telkomsel</t>
+          <t>myxl</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>2496757</v>
+        <v>409801</v>
       </c>
       <c r="C3" t="n">
-        <v>2496796</v>
+        <v>409739</v>
       </c>
       <c r="D3" t="n">
-        <v>-39</v>
+        <v>62</v>
       </c>
       <c r="E3" t="n">
-        <v>-0.0016</v>
+        <v>0.0151</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily follower scan: 2026-09-17
</commit_message>
<xml_diff>
--- a/daily_report.xlsx
+++ b/daily_report.xlsx
@@ -446,39 +446,39 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>telkomsel</t>
+          <t>myxl</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>2496649</v>
+        <v>409901</v>
       </c>
       <c r="C2" t="n">
-        <v>2496757</v>
+        <v>409801</v>
       </c>
       <c r="D2" t="n">
-        <v>-108</v>
+        <v>100</v>
       </c>
       <c r="E2" t="n">
-        <v>-0.0043</v>
+        <v>0.0244</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>myxl</t>
+          <t>telkomsel</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>409801</v>
+        <v>2496640</v>
       </c>
       <c r="C3" t="n">
-        <v>409739</v>
+        <v>2496649</v>
       </c>
       <c r="D3" t="n">
-        <v>62</v>
+        <v>-9</v>
       </c>
       <c r="E3" t="n">
-        <v>0.0151</v>
+        <v>-0.0004</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily follower scan: 2026-09-18
</commit_message>
<xml_diff>
--- a/daily_report.xlsx
+++ b/daily_report.xlsx
@@ -450,16 +450,16 @@
         </is>
       </c>
       <c r="B2" t="n">
+        <v>410002</v>
+      </c>
+      <c r="C2" t="n">
         <v>409901</v>
       </c>
-      <c r="C2" t="n">
-        <v>409801</v>
-      </c>
       <c r="D2" t="n">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="E2" t="n">
-        <v>0.0244</v>
+        <v>0.0246</v>
       </c>
     </row>
     <row r="3">
@@ -469,16 +469,16 @@
         </is>
       </c>
       <c r="B3" t="n">
+        <v>2496621</v>
+      </c>
+      <c r="C3" t="n">
         <v>2496640</v>
       </c>
-      <c r="C3" t="n">
-        <v>2496649</v>
-      </c>
       <c r="D3" t="n">
-        <v>-9</v>
+        <v>-19</v>
       </c>
       <c r="E3" t="n">
-        <v>-0.0004</v>
+        <v>-0.0008</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily follower scan: 2026-09-19
</commit_message>
<xml_diff>
--- a/daily_report.xlsx
+++ b/daily_report.xlsx
@@ -450,16 +450,16 @@
         </is>
       </c>
       <c r="B2" t="n">
+        <v>410057</v>
+      </c>
+      <c r="C2" t="n">
         <v>410002</v>
       </c>
-      <c r="C2" t="n">
-        <v>409901</v>
-      </c>
       <c r="D2" t="n">
-        <v>101</v>
+        <v>55</v>
       </c>
       <c r="E2" t="n">
-        <v>0.0246</v>
+        <v>0.0134</v>
       </c>
     </row>
     <row r="3">
@@ -469,16 +469,16 @@
         </is>
       </c>
       <c r="B3" t="n">
+        <v>2496591</v>
+      </c>
+      <c r="C3" t="n">
         <v>2496621</v>
       </c>
-      <c r="C3" t="n">
-        <v>2496640</v>
-      </c>
       <c r="D3" t="n">
-        <v>-19</v>
+        <v>-30</v>
       </c>
       <c r="E3" t="n">
-        <v>-0.0008</v>
+        <v>-0.0012</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily follower scan: 2026-09-20
</commit_message>
<xml_diff>
--- a/daily_report.xlsx
+++ b/daily_report.xlsx
@@ -450,16 +450,16 @@
         </is>
       </c>
       <c r="B2" t="n">
+        <v>410139</v>
+      </c>
+      <c r="C2" t="n">
         <v>410057</v>
       </c>
-      <c r="C2" t="n">
-        <v>410002</v>
-      </c>
       <c r="D2" t="n">
-        <v>55</v>
+        <v>82</v>
       </c>
       <c r="E2" t="n">
-        <v>0.0134</v>
+        <v>0.02</v>
       </c>
     </row>
     <row r="3">
@@ -469,16 +469,16 @@
         </is>
       </c>
       <c r="B3" t="n">
+        <v>2496547</v>
+      </c>
+      <c r="C3" t="n">
         <v>2496591</v>
       </c>
-      <c r="C3" t="n">
-        <v>2496621</v>
-      </c>
       <c r="D3" t="n">
-        <v>-30</v>
+        <v>-44</v>
       </c>
       <c r="E3" t="n">
-        <v>-0.0012</v>
+        <v>-0.0018</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily follower scan: 2026-09-21
</commit_message>
<xml_diff>
--- a/daily_report.xlsx
+++ b/daily_report.xlsx
@@ -450,16 +450,16 @@
         </is>
       </c>
       <c r="B2" t="n">
+        <v>410244</v>
+      </c>
+      <c r="C2" t="n">
         <v>410139</v>
       </c>
-      <c r="C2" t="n">
-        <v>410057</v>
-      </c>
       <c r="D2" t="n">
-        <v>82</v>
+        <v>105</v>
       </c>
       <c r="E2" t="n">
-        <v>0.02</v>
+        <v>0.0256</v>
       </c>
     </row>
     <row r="3">
@@ -469,16 +469,16 @@
         </is>
       </c>
       <c r="B3" t="n">
+        <v>2496536</v>
+      </c>
+      <c r="C3" t="n">
         <v>2496547</v>
       </c>
-      <c r="C3" t="n">
-        <v>2496591</v>
-      </c>
       <c r="D3" t="n">
-        <v>-44</v>
+        <v>-11</v>
       </c>
       <c r="E3" t="n">
-        <v>-0.0018</v>
+        <v>-0.0004</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily follower scan: 2026-09-22
</commit_message>
<xml_diff>
--- a/daily_report.xlsx
+++ b/daily_report.xlsx
@@ -446,39 +446,39 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>myxl</t>
+          <t>telkomsel</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>410244</v>
+        <v>2496472</v>
       </c>
       <c r="C2" t="n">
-        <v>410139</v>
+        <v>2496536</v>
       </c>
       <c r="D2" t="n">
-        <v>105</v>
+        <v>-64</v>
       </c>
       <c r="E2" t="n">
-        <v>0.0256</v>
+        <v>-0.0026</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>telkomsel</t>
+          <t>myxl</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>2496536</v>
+        <v>410305</v>
       </c>
       <c r="C3" t="n">
-        <v>2496547</v>
+        <v>410244</v>
       </c>
       <c r="D3" t="n">
-        <v>-11</v>
+        <v>61</v>
       </c>
       <c r="E3" t="n">
-        <v>-0.0004</v>
+        <v>0.0149</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily follower scan: 2026-09-23
</commit_message>
<xml_diff>
--- a/daily_report.xlsx
+++ b/daily_report.xlsx
@@ -446,39 +446,39 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>telkomsel</t>
+          <t>myxl</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>2496472</v>
+        <v>410358</v>
       </c>
       <c r="C2" t="n">
-        <v>2496536</v>
+        <v>410305</v>
       </c>
       <c r="D2" t="n">
-        <v>-64</v>
+        <v>53</v>
       </c>
       <c r="E2" t="n">
-        <v>-0.0026</v>
+        <v>0.0129</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>myxl</t>
+          <t>telkomsel</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>410305</v>
+        <v>2496444</v>
       </c>
       <c r="C3" t="n">
-        <v>410244</v>
+        <v>2496472</v>
       </c>
       <c r="D3" t="n">
-        <v>61</v>
+        <v>-28</v>
       </c>
       <c r="E3" t="n">
-        <v>0.0149</v>
+        <v>-0.0011</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily follower scan: 2026-09-24
</commit_message>
<xml_diff>
--- a/daily_report.xlsx
+++ b/daily_report.xlsx
@@ -446,39 +446,39 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>myxl</t>
+          <t>telkomsel</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>410358</v>
+        <v>2496356</v>
       </c>
       <c r="C2" t="n">
-        <v>410305</v>
+        <v>2496444</v>
       </c>
       <c r="D2" t="n">
-        <v>53</v>
+        <v>-88</v>
       </c>
       <c r="E2" t="n">
-        <v>0.0129</v>
+        <v>-0.0035</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>telkomsel</t>
+          <t>myxl</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>2496444</v>
+        <v>410422</v>
       </c>
       <c r="C3" t="n">
-        <v>2496472</v>
+        <v>410358</v>
       </c>
       <c r="D3" t="n">
-        <v>-28</v>
+        <v>64</v>
       </c>
       <c r="E3" t="n">
-        <v>-0.0011</v>
+        <v>0.0156</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily follower scan: 2026-09-25
</commit_message>
<xml_diff>
--- a/daily_report.xlsx
+++ b/daily_report.xlsx
@@ -446,39 +446,39 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>telkomsel</t>
+          <t>myxl</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>2496356</v>
+        <v>410501</v>
       </c>
       <c r="C2" t="n">
-        <v>2496444</v>
+        <v>410422</v>
       </c>
       <c r="D2" t="n">
-        <v>-88</v>
+        <v>79</v>
       </c>
       <c r="E2" t="n">
-        <v>-0.0035</v>
+        <v>0.0192</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>myxl</t>
+          <t>telkomsel</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>410422</v>
+        <v>2496354</v>
       </c>
       <c r="C3" t="n">
-        <v>410358</v>
+        <v>2496356</v>
       </c>
       <c r="D3" t="n">
-        <v>64</v>
+        <v>-2</v>
       </c>
       <c r="E3" t="n">
-        <v>0.0156</v>
+        <v>-0.0001</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily follower scan: 2026-09-26
</commit_message>
<xml_diff>
--- a/daily_report.xlsx
+++ b/daily_report.xlsx
@@ -450,16 +450,16 @@
         </is>
       </c>
       <c r="B2" t="n">
+        <v>410672</v>
+      </c>
+      <c r="C2" t="n">
         <v>410501</v>
       </c>
-      <c r="C2" t="n">
-        <v>410422</v>
-      </c>
       <c r="D2" t="n">
-        <v>79</v>
+        <v>171</v>
       </c>
       <c r="E2" t="n">
-        <v>0.0192</v>
+        <v>0.0417</v>
       </c>
     </row>
     <row r="3">
@@ -469,16 +469,16 @@
         </is>
       </c>
       <c r="B3" t="n">
+        <v>2496360</v>
+      </c>
+      <c r="C3" t="n">
         <v>2496354</v>
       </c>
-      <c r="C3" t="n">
-        <v>2496356</v>
-      </c>
       <c r="D3" t="n">
-        <v>-2</v>
+        <v>6</v>
       </c>
       <c r="E3" t="n">
-        <v>-0.0001</v>
+        <v>0.0002</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily follower scan: 2026-09-27
</commit_message>
<xml_diff>
--- a/daily_report.xlsx
+++ b/daily_report.xlsx
@@ -450,16 +450,16 @@
         </is>
       </c>
       <c r="B2" t="n">
+        <v>410789</v>
+      </c>
+      <c r="C2" t="n">
         <v>410672</v>
       </c>
-      <c r="C2" t="n">
-        <v>410501</v>
-      </c>
       <c r="D2" t="n">
-        <v>171</v>
+        <v>117</v>
       </c>
       <c r="E2" t="n">
-        <v>0.0417</v>
+        <v>0.0285</v>
       </c>
     </row>
     <row r="3">
@@ -469,16 +469,16 @@
         </is>
       </c>
       <c r="B3" t="n">
+        <v>2496350</v>
+      </c>
+      <c r="C3" t="n">
         <v>2496360</v>
       </c>
-      <c r="C3" t="n">
-        <v>2496354</v>
-      </c>
       <c r="D3" t="n">
-        <v>6</v>
+        <v>-10</v>
       </c>
       <c r="E3" t="n">
-        <v>0.0002</v>
+        <v>-0.0004</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily follower scan: 2026-09-28
</commit_message>
<xml_diff>
--- a/daily_report.xlsx
+++ b/daily_report.xlsx
@@ -450,16 +450,16 @@
         </is>
       </c>
       <c r="B2" t="n">
+        <v>410897</v>
+      </c>
+      <c r="C2" t="n">
         <v>410789</v>
       </c>
-      <c r="C2" t="n">
-        <v>410672</v>
-      </c>
       <c r="D2" t="n">
-        <v>117</v>
+        <v>108</v>
       </c>
       <c r="E2" t="n">
-        <v>0.0285</v>
+        <v>0.0263</v>
       </c>
     </row>
     <row r="3">
@@ -469,16 +469,16 @@
         </is>
       </c>
       <c r="B3" t="n">
+        <v>2496330</v>
+      </c>
+      <c r="C3" t="n">
         <v>2496350</v>
       </c>
-      <c r="C3" t="n">
-        <v>2496360</v>
-      </c>
       <c r="D3" t="n">
-        <v>-10</v>
+        <v>-20</v>
       </c>
       <c r="E3" t="n">
-        <v>-0.0004</v>
+        <v>-0.0008</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily follower scan: 2026-09-29
</commit_message>
<xml_diff>
--- a/daily_report.xlsx
+++ b/daily_report.xlsx
@@ -450,16 +450,16 @@
         </is>
       </c>
       <c r="B2" t="n">
+        <v>411001</v>
+      </c>
+      <c r="C2" t="n">
         <v>410897</v>
       </c>
-      <c r="C2" t="n">
-        <v>410789</v>
-      </c>
       <c r="D2" t="n">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="E2" t="n">
-        <v>0.0263</v>
+        <v>0.0253</v>
       </c>
     </row>
     <row r="3">
@@ -469,16 +469,16 @@
         </is>
       </c>
       <c r="B3" t="n">
+        <v>2496339</v>
+      </c>
+      <c r="C3" t="n">
         <v>2496330</v>
       </c>
-      <c r="C3" t="n">
-        <v>2496350</v>
-      </c>
       <c r="D3" t="n">
-        <v>-20</v>
+        <v>9</v>
       </c>
       <c r="E3" t="n">
-        <v>-0.0008</v>
+        <v>0.0004</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily follower scan: 2026-09-30
</commit_message>
<xml_diff>
--- a/daily_report.xlsx
+++ b/daily_report.xlsx
@@ -450,16 +450,16 @@
         </is>
       </c>
       <c r="B2" t="n">
+        <v>411125</v>
+      </c>
+      <c r="C2" t="n">
         <v>411001</v>
       </c>
-      <c r="C2" t="n">
-        <v>410897</v>
-      </c>
       <c r="D2" t="n">
-        <v>104</v>
+        <v>124</v>
       </c>
       <c r="E2" t="n">
-        <v>0.0253</v>
+        <v>0.0302</v>
       </c>
     </row>
     <row r="3">
@@ -469,16 +469,16 @@
         </is>
       </c>
       <c r="B3" t="n">
+        <v>2496347</v>
+      </c>
+      <c r="C3" t="n">
         <v>2496339</v>
       </c>
-      <c r="C3" t="n">
-        <v>2496330</v>
-      </c>
       <c r="D3" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E3" t="n">
-        <v>0.0004</v>
+        <v>0.0003</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily follower scan: 2026-10-01
</commit_message>
<xml_diff>
--- a/daily_report.xlsx
+++ b/daily_report.xlsx
@@ -450,16 +450,16 @@
         </is>
       </c>
       <c r="B2" t="n">
+        <v>411269</v>
+      </c>
+      <c r="C2" t="n">
         <v>411125</v>
       </c>
-      <c r="C2" t="n">
-        <v>411001</v>
-      </c>
       <c r="D2" t="n">
-        <v>124</v>
+        <v>144</v>
       </c>
       <c r="E2" t="n">
-        <v>0.0302</v>
+        <v>0.035</v>
       </c>
     </row>
     <row r="3">
@@ -469,16 +469,16 @@
         </is>
       </c>
       <c r="B3" t="n">
+        <v>2496387</v>
+      </c>
+      <c r="C3" t="n">
         <v>2496347</v>
       </c>
-      <c r="C3" t="n">
-        <v>2496339</v>
-      </c>
       <c r="D3" t="n">
-        <v>8</v>
+        <v>40</v>
       </c>
       <c r="E3" t="n">
-        <v>0.0003</v>
+        <v>0.0016</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily follower scan: 2026-10-02
</commit_message>
<xml_diff>
--- a/daily_report.xlsx
+++ b/daily_report.xlsx
@@ -450,16 +450,16 @@
         </is>
       </c>
       <c r="B2" t="n">
+        <v>411435</v>
+      </c>
+      <c r="C2" t="n">
         <v>411269</v>
       </c>
-      <c r="C2" t="n">
-        <v>411125</v>
-      </c>
       <c r="D2" t="n">
-        <v>144</v>
+        <v>166</v>
       </c>
       <c r="E2" t="n">
-        <v>0.035</v>
+        <v>0.0404</v>
       </c>
     </row>
     <row r="3">
@@ -469,16 +469,16 @@
         </is>
       </c>
       <c r="B3" t="n">
+        <v>2496370</v>
+      </c>
+      <c r="C3" t="n">
         <v>2496387</v>
       </c>
-      <c r="C3" t="n">
-        <v>2496347</v>
-      </c>
       <c r="D3" t="n">
-        <v>40</v>
+        <v>-17</v>
       </c>
       <c r="E3" t="n">
-        <v>0.0016</v>
+        <v>-0.0007</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily follower scan: 2026-10-03
</commit_message>
<xml_diff>
--- a/daily_report.xlsx
+++ b/daily_report.xlsx
@@ -450,16 +450,16 @@
         </is>
       </c>
       <c r="B2" t="n">
+        <v>411551</v>
+      </c>
+      <c r="C2" t="n">
         <v>411435</v>
       </c>
-      <c r="C2" t="n">
-        <v>411269</v>
-      </c>
       <c r="D2" t="n">
-        <v>166</v>
+        <v>116</v>
       </c>
       <c r="E2" t="n">
-        <v>0.0404</v>
+        <v>0.0282</v>
       </c>
     </row>
     <row r="3">
@@ -469,16 +469,16 @@
         </is>
       </c>
       <c r="B3" t="n">
+        <v>2496297</v>
+      </c>
+      <c r="C3" t="n">
         <v>2496370</v>
       </c>
-      <c r="C3" t="n">
-        <v>2496387</v>
-      </c>
       <c r="D3" t="n">
-        <v>-17</v>
+        <v>-73</v>
       </c>
       <c r="E3" t="n">
-        <v>-0.0007</v>
+        <v>-0.0029</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily follower scan: 2026-10-04
</commit_message>
<xml_diff>
--- a/daily_report.xlsx
+++ b/daily_report.xlsx
@@ -450,16 +450,16 @@
         </is>
       </c>
       <c r="B2" t="n">
+        <v>411733</v>
+      </c>
+      <c r="C2" t="n">
         <v>411551</v>
       </c>
-      <c r="C2" t="n">
-        <v>411435</v>
-      </c>
       <c r="D2" t="n">
-        <v>116</v>
+        <v>182</v>
       </c>
       <c r="E2" t="n">
-        <v>0.0282</v>
+        <v>0.0442</v>
       </c>
     </row>
     <row r="3">
@@ -469,16 +469,16 @@
         </is>
       </c>
       <c r="B3" t="n">
+        <v>2496241</v>
+      </c>
+      <c r="C3" t="n">
         <v>2496297</v>
       </c>
-      <c r="C3" t="n">
-        <v>2496370</v>
-      </c>
       <c r="D3" t="n">
-        <v>-73</v>
+        <v>-56</v>
       </c>
       <c r="E3" t="n">
-        <v>-0.0029</v>
+        <v>-0.0022</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily follower scan: 2026-10-05
</commit_message>
<xml_diff>
--- a/daily_report.xlsx
+++ b/daily_report.xlsx
@@ -450,16 +450,16 @@
         </is>
       </c>
       <c r="B2" t="n">
+        <v>411908</v>
+      </c>
+      <c r="C2" t="n">
         <v>411733</v>
       </c>
-      <c r="C2" t="n">
-        <v>411551</v>
-      </c>
       <c r="D2" t="n">
-        <v>182</v>
+        <v>175</v>
       </c>
       <c r="E2" t="n">
-        <v>0.0442</v>
+        <v>0.0425</v>
       </c>
     </row>
     <row r="3">
@@ -469,16 +469,16 @@
         </is>
       </c>
       <c r="B3" t="n">
+        <v>2496232</v>
+      </c>
+      <c r="C3" t="n">
         <v>2496241</v>
       </c>
-      <c r="C3" t="n">
-        <v>2496297</v>
-      </c>
       <c r="D3" t="n">
-        <v>-56</v>
+        <v>-9</v>
       </c>
       <c r="E3" t="n">
-        <v>-0.0022</v>
+        <v>-0.0004</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily follower scan: 2026-10-06
</commit_message>
<xml_diff>
--- a/daily_report.xlsx
+++ b/daily_report.xlsx
@@ -450,16 +450,16 @@
         </is>
       </c>
       <c r="B2" t="n">
+        <v>412055</v>
+      </c>
+      <c r="C2" t="n">
         <v>411908</v>
       </c>
-      <c r="C2" t="n">
-        <v>411733</v>
-      </c>
       <c r="D2" t="n">
-        <v>175</v>
+        <v>147</v>
       </c>
       <c r="E2" t="n">
-        <v>0.0425</v>
+        <v>0.0357</v>
       </c>
     </row>
     <row r="3">
@@ -469,16 +469,16 @@
         </is>
       </c>
       <c r="B3" t="n">
+        <v>2496180</v>
+      </c>
+      <c r="C3" t="n">
         <v>2496232</v>
       </c>
-      <c r="C3" t="n">
-        <v>2496241</v>
-      </c>
       <c r="D3" t="n">
-        <v>-9</v>
+        <v>-52</v>
       </c>
       <c r="E3" t="n">
-        <v>-0.0004</v>
+        <v>-0.0021</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily follower scan: 2026-10-07
</commit_message>
<xml_diff>
--- a/daily_report.xlsx
+++ b/daily_report.xlsx
@@ -450,16 +450,16 @@
         </is>
       </c>
       <c r="B2" t="n">
+        <v>412200</v>
+      </c>
+      <c r="C2" t="n">
         <v>412055</v>
       </c>
-      <c r="C2" t="n">
-        <v>411908</v>
-      </c>
       <c r="D2" t="n">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="E2" t="n">
-        <v>0.0357</v>
+        <v>0.0352</v>
       </c>
     </row>
     <row r="3">
@@ -469,16 +469,16 @@
         </is>
       </c>
       <c r="B3" t="n">
+        <v>2496150</v>
+      </c>
+      <c r="C3" t="n">
         <v>2496180</v>
       </c>
-      <c r="C3" t="n">
-        <v>2496232</v>
-      </c>
       <c r="D3" t="n">
-        <v>-52</v>
+        <v>-30</v>
       </c>
       <c r="E3" t="n">
-        <v>-0.0021</v>
+        <v>-0.0012</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily follower scan: 2026-10-08
</commit_message>
<xml_diff>
--- a/daily_report.xlsx
+++ b/daily_report.xlsx
@@ -450,16 +450,16 @@
         </is>
       </c>
       <c r="B2" t="n">
+        <v>412384</v>
+      </c>
+      <c r="C2" t="n">
         <v>412200</v>
       </c>
-      <c r="C2" t="n">
-        <v>412055</v>
-      </c>
       <c r="D2" t="n">
-        <v>145</v>
+        <v>184</v>
       </c>
       <c r="E2" t="n">
-        <v>0.0352</v>
+        <v>0.0446</v>
       </c>
     </row>
     <row r="3">
@@ -469,16 +469,16 @@
         </is>
       </c>
       <c r="B3" t="n">
+        <v>2496076</v>
+      </c>
+      <c r="C3" t="n">
         <v>2496150</v>
       </c>
-      <c r="C3" t="n">
-        <v>2496180</v>
-      </c>
       <c r="D3" t="n">
-        <v>-30</v>
+        <v>-74</v>
       </c>
       <c r="E3" t="n">
-        <v>-0.0012</v>
+        <v>-0.003</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily follower scan: 2026-10-09
</commit_message>
<xml_diff>
--- a/daily_report.xlsx
+++ b/daily_report.xlsx
@@ -450,16 +450,16 @@
         </is>
       </c>
       <c r="B2" t="n">
+        <v>412543</v>
+      </c>
+      <c r="C2" t="n">
         <v>412384</v>
       </c>
-      <c r="C2" t="n">
-        <v>412200</v>
-      </c>
       <c r="D2" t="n">
-        <v>184</v>
+        <v>159</v>
       </c>
       <c r="E2" t="n">
-        <v>0.0446</v>
+        <v>0.0386</v>
       </c>
     </row>
     <row r="3">
@@ -469,16 +469,16 @@
         </is>
       </c>
       <c r="B3" t="n">
+        <v>2496050</v>
+      </c>
+      <c r="C3" t="n">
         <v>2496076</v>
       </c>
-      <c r="C3" t="n">
-        <v>2496150</v>
-      </c>
       <c r="D3" t="n">
-        <v>-74</v>
+        <v>-26</v>
       </c>
       <c r="E3" t="n">
-        <v>-0.003</v>
+        <v>-0.001</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily follower scan: 2026-10-10
</commit_message>
<xml_diff>
--- a/daily_report.xlsx
+++ b/daily_report.xlsx
@@ -450,16 +450,16 @@
         </is>
       </c>
       <c r="B2" t="n">
+        <v>412639</v>
+      </c>
+      <c r="C2" t="n">
         <v>412543</v>
       </c>
-      <c r="C2" t="n">
-        <v>412384</v>
-      </c>
       <c r="D2" t="n">
-        <v>159</v>
+        <v>96</v>
       </c>
       <c r="E2" t="n">
-        <v>0.0386</v>
+        <v>0.0233</v>
       </c>
     </row>
     <row r="3">
@@ -469,16 +469,16 @@
         </is>
       </c>
       <c r="B3" t="n">
+        <v>2496073</v>
+      </c>
+      <c r="C3" t="n">
         <v>2496050</v>
       </c>
-      <c r="C3" t="n">
-        <v>2496076</v>
-      </c>
       <c r="D3" t="n">
-        <v>-26</v>
+        <v>23</v>
       </c>
       <c r="E3" t="n">
-        <v>-0.001</v>
+        <v>0.0009</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily follower scan: 2026-10-11
</commit_message>
<xml_diff>
--- a/daily_report.xlsx
+++ b/daily_report.xlsx
@@ -450,16 +450,16 @@
         </is>
       </c>
       <c r="B2" t="n">
+        <v>412785</v>
+      </c>
+      <c r="C2" t="n">
         <v>412639</v>
       </c>
-      <c r="C2" t="n">
-        <v>412543</v>
-      </c>
       <c r="D2" t="n">
-        <v>96</v>
+        <v>146</v>
       </c>
       <c r="E2" t="n">
-        <v>0.0233</v>
+        <v>0.0354</v>
       </c>
     </row>
     <row r="3">
@@ -469,16 +469,16 @@
         </is>
       </c>
       <c r="B3" t="n">
+        <v>2496159</v>
+      </c>
+      <c r="C3" t="n">
         <v>2496073</v>
       </c>
-      <c r="C3" t="n">
-        <v>2496050</v>
-      </c>
       <c r="D3" t="n">
-        <v>23</v>
+        <v>86</v>
       </c>
       <c r="E3" t="n">
-        <v>0.0009</v>
+        <v>0.0034</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily follower scan: 2026-10-12
</commit_message>
<xml_diff>
--- a/daily_report.xlsx
+++ b/daily_report.xlsx
@@ -450,16 +450,16 @@
         </is>
       </c>
       <c r="B2" t="n">
+        <v>412970</v>
+      </c>
+      <c r="C2" t="n">
         <v>412785</v>
       </c>
-      <c r="C2" t="n">
-        <v>412639</v>
-      </c>
       <c r="D2" t="n">
-        <v>146</v>
+        <v>185</v>
       </c>
       <c r="E2" t="n">
-        <v>0.0354</v>
+        <v>0.0448</v>
       </c>
     </row>
     <row r="3">
@@ -469,16 +469,16 @@
         </is>
       </c>
       <c r="B3" t="n">
+        <v>2496121</v>
+      </c>
+      <c r="C3" t="n">
         <v>2496159</v>
       </c>
-      <c r="C3" t="n">
-        <v>2496073</v>
-      </c>
       <c r="D3" t="n">
-        <v>86</v>
+        <v>-38</v>
       </c>
       <c r="E3" t="n">
-        <v>0.0034</v>
+        <v>-0.0015</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily follower scan: 2026-10-13
</commit_message>
<xml_diff>
--- a/daily_report.xlsx
+++ b/daily_report.xlsx
@@ -446,39 +446,39 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>myxl</t>
+          <t>telkomsel</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>412970</v>
+        <v>2496341</v>
       </c>
       <c r="C2" t="n">
-        <v>412785</v>
+        <v>2496121</v>
       </c>
       <c r="D2" t="n">
-        <v>185</v>
+        <v>220</v>
       </c>
       <c r="E2" t="n">
-        <v>0.0448</v>
+        <v>0.008800000000000001</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>telkomsel</t>
+          <t>myxl</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>2496121</v>
+        <v>413173</v>
       </c>
       <c r="C3" t="n">
-        <v>2496159</v>
+        <v>412970</v>
       </c>
       <c r="D3" t="n">
-        <v>-38</v>
+        <v>203</v>
       </c>
       <c r="E3" t="n">
-        <v>-0.0015</v>
+        <v>0.0492</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily follower scan: 2026-10-14
</commit_message>
<xml_diff>
--- a/daily_report.xlsx
+++ b/daily_report.xlsx
@@ -446,39 +446,39 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>telkomsel</t>
+          <t>myxl</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>2496341</v>
+        <v>413372</v>
       </c>
       <c r="C2" t="n">
-        <v>2496121</v>
+        <v>413173</v>
       </c>
       <c r="D2" t="n">
-        <v>220</v>
+        <v>199</v>
       </c>
       <c r="E2" t="n">
-        <v>0.008800000000000001</v>
+        <v>0.0482</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>myxl</t>
+          <t>telkomsel</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>413173</v>
+        <v>2496500</v>
       </c>
       <c r="C3" t="n">
-        <v>412970</v>
+        <v>2496341</v>
       </c>
       <c r="D3" t="n">
-        <v>203</v>
+        <v>159</v>
       </c>
       <c r="E3" t="n">
-        <v>0.0492</v>
+        <v>0.0064</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily follower scan: 2026-10-15
</commit_message>
<xml_diff>
--- a/daily_report.xlsx
+++ b/daily_report.xlsx
@@ -450,16 +450,16 @@
         </is>
       </c>
       <c r="B2" t="n">
+        <v>413490</v>
+      </c>
+      <c r="C2" t="n">
         <v>413372</v>
       </c>
-      <c r="C2" t="n">
-        <v>413173</v>
-      </c>
       <c r="D2" t="n">
-        <v>199</v>
+        <v>118</v>
       </c>
       <c r="E2" t="n">
-        <v>0.0482</v>
+        <v>0.0285</v>
       </c>
     </row>
     <row r="3">
@@ -469,16 +469,16 @@
         </is>
       </c>
       <c r="B3" t="n">
+        <v>2496498</v>
+      </c>
+      <c r="C3" t="n">
         <v>2496500</v>
       </c>
-      <c r="C3" t="n">
-        <v>2496341</v>
-      </c>
       <c r="D3" t="n">
-        <v>159</v>
+        <v>-2</v>
       </c>
       <c r="E3" t="n">
-        <v>0.0064</v>
+        <v>-0.0001</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily follower scan: 2026-10-16
</commit_message>
<xml_diff>
--- a/daily_report.xlsx
+++ b/daily_report.xlsx
@@ -450,16 +450,16 @@
         </is>
       </c>
       <c r="B2" t="n">
+        <v>413544</v>
+      </c>
+      <c r="C2" t="n">
         <v>413490</v>
       </c>
-      <c r="C2" t="n">
-        <v>413372</v>
-      </c>
       <c r="D2" t="n">
-        <v>118</v>
+        <v>54</v>
       </c>
       <c r="E2" t="n">
-        <v>0.0285</v>
+        <v>0.0131</v>
       </c>
     </row>
     <row r="3">
@@ -469,16 +469,16 @@
         </is>
       </c>
       <c r="B3" t="n">
+        <v>2496456</v>
+      </c>
+      <c r="C3" t="n">
         <v>2496498</v>
       </c>
-      <c r="C3" t="n">
-        <v>2496500</v>
-      </c>
       <c r="D3" t="n">
-        <v>-2</v>
+        <v>-42</v>
       </c>
       <c r="E3" t="n">
-        <v>-0.0001</v>
+        <v>-0.0017</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily follower scan: 2026-10-17
</commit_message>
<xml_diff>
--- a/daily_report.xlsx
+++ b/daily_report.xlsx
@@ -450,16 +450,16 @@
         </is>
       </c>
       <c r="B2" t="n">
+        <v>413669</v>
+      </c>
+      <c r="C2" t="n">
         <v>413544</v>
       </c>
-      <c r="C2" t="n">
-        <v>413490</v>
-      </c>
       <c r="D2" t="n">
-        <v>54</v>
+        <v>125</v>
       </c>
       <c r="E2" t="n">
-        <v>0.0131</v>
+        <v>0.0302</v>
       </c>
     </row>
     <row r="3">
@@ -469,16 +469,16 @@
         </is>
       </c>
       <c r="B3" t="n">
+        <v>2496545</v>
+      </c>
+      <c r="C3" t="n">
         <v>2496456</v>
       </c>
-      <c r="C3" t="n">
-        <v>2496498</v>
-      </c>
       <c r="D3" t="n">
-        <v>-42</v>
+        <v>89</v>
       </c>
       <c r="E3" t="n">
-        <v>-0.0017</v>
+        <v>0.0036</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily follower scan: 2026-10-18
</commit_message>
<xml_diff>
--- a/daily_report.xlsx
+++ b/daily_report.xlsx
@@ -450,16 +450,16 @@
         </is>
       </c>
       <c r="B2" t="n">
+        <v>413807</v>
+      </c>
+      <c r="C2" t="n">
         <v>413669</v>
       </c>
-      <c r="C2" t="n">
-        <v>413544</v>
-      </c>
       <c r="D2" t="n">
-        <v>125</v>
+        <v>138</v>
       </c>
       <c r="E2" t="n">
-        <v>0.0302</v>
+        <v>0.0334</v>
       </c>
     </row>
     <row r="3">
@@ -469,16 +469,16 @@
         </is>
       </c>
       <c r="B3" t="n">
+        <v>2496587</v>
+      </c>
+      <c r="C3" t="n">
         <v>2496545</v>
       </c>
-      <c r="C3" t="n">
-        <v>2496456</v>
-      </c>
       <c r="D3" t="n">
-        <v>89</v>
+        <v>42</v>
       </c>
       <c r="E3" t="n">
-        <v>0.0036</v>
+        <v>0.0017</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily follower scan: 2026-10-19
</commit_message>
<xml_diff>
--- a/daily_report.xlsx
+++ b/daily_report.xlsx
@@ -446,39 +446,39 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>myxl</t>
+          <t>telkomsel</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>413807</v>
+        <v>2496713</v>
       </c>
       <c r="C2" t="n">
-        <v>413669</v>
+        <v>2496587</v>
       </c>
       <c r="D2" t="n">
-        <v>138</v>
+        <v>126</v>
       </c>
       <c r="E2" t="n">
-        <v>0.0334</v>
+        <v>0.005</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>telkomsel</t>
+          <t>myxl</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>2496587</v>
+        <v>413890</v>
       </c>
       <c r="C3" t="n">
-        <v>2496545</v>
+        <v>413807</v>
       </c>
       <c r="D3" t="n">
-        <v>42</v>
+        <v>83</v>
       </c>
       <c r="E3" t="n">
-        <v>0.0017</v>
+        <v>0.0201</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily follower scan: 2026-10-20
</commit_message>
<xml_diff>
--- a/daily_report.xlsx
+++ b/daily_report.xlsx
@@ -446,39 +446,39 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>telkomsel</t>
+          <t>myxl</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>2496713</v>
+        <v>413986</v>
       </c>
       <c r="C2" t="n">
-        <v>2496587</v>
+        <v>413890</v>
       </c>
       <c r="D2" t="n">
-        <v>126</v>
+        <v>96</v>
       </c>
       <c r="E2" t="n">
-        <v>0.005</v>
+        <v>0.0232</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>myxl</t>
+          <t>telkomsel</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>413890</v>
+        <v>2496806</v>
       </c>
       <c r="C3" t="n">
-        <v>413807</v>
+        <v>2496713</v>
       </c>
       <c r="D3" t="n">
-        <v>83</v>
+        <v>93</v>
       </c>
       <c r="E3" t="n">
-        <v>0.0201</v>
+        <v>0.0037</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily follower scan: 2026-10-21
</commit_message>
<xml_diff>
--- a/daily_report.xlsx
+++ b/daily_report.xlsx
@@ -450,16 +450,16 @@
         </is>
       </c>
       <c r="B2" t="n">
+        <v>414076</v>
+      </c>
+      <c r="C2" t="n">
         <v>413986</v>
       </c>
-      <c r="C2" t="n">
-        <v>413890</v>
-      </c>
       <c r="D2" t="n">
-        <v>96</v>
+        <v>90</v>
       </c>
       <c r="E2" t="n">
-        <v>0.0232</v>
+        <v>0.0217</v>
       </c>
     </row>
     <row r="3">
@@ -469,16 +469,16 @@
         </is>
       </c>
       <c r="B3" t="n">
+        <v>2496881</v>
+      </c>
+      <c r="C3" t="n">
         <v>2496806</v>
       </c>
-      <c r="C3" t="n">
-        <v>2496713</v>
-      </c>
       <c r="D3" t="n">
-        <v>93</v>
+        <v>75</v>
       </c>
       <c r="E3" t="n">
-        <v>0.0037</v>
+        <v>0.003</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily follower scan: 2026-10-22
</commit_message>
<xml_diff>
--- a/daily_report.xlsx
+++ b/daily_report.xlsx
@@ -450,16 +450,16 @@
         </is>
       </c>
       <c r="B2" t="n">
+        <v>414171</v>
+      </c>
+      <c r="C2" t="n">
         <v>414076</v>
       </c>
-      <c r="C2" t="n">
-        <v>413986</v>
-      </c>
       <c r="D2" t="n">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="E2" t="n">
-        <v>0.0217</v>
+        <v>0.0229</v>
       </c>
     </row>
     <row r="3">
@@ -469,16 +469,16 @@
         </is>
       </c>
       <c r="B3" t="n">
+        <v>2496926</v>
+      </c>
+      <c r="C3" t="n">
         <v>2496881</v>
       </c>
-      <c r="C3" t="n">
-        <v>2496806</v>
-      </c>
       <c r="D3" t="n">
-        <v>75</v>
+        <v>45</v>
       </c>
       <c r="E3" t="n">
-        <v>0.003</v>
+        <v>0.0018</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily follower scan: 2026-10-23
</commit_message>
<xml_diff>
--- a/daily_report.xlsx
+++ b/daily_report.xlsx
@@ -446,39 +446,39 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>myxl</t>
+          <t>telkomsel</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>414171</v>
+        <v>2497091</v>
       </c>
       <c r="C2" t="n">
-        <v>414076</v>
+        <v>2496926</v>
       </c>
       <c r="D2" t="n">
-        <v>95</v>
+        <v>165</v>
       </c>
       <c r="E2" t="n">
-        <v>0.0229</v>
+        <v>0.0066</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>telkomsel</t>
+          <t>myxl</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>2496926</v>
+        <v>414256</v>
       </c>
       <c r="C3" t="n">
-        <v>2496881</v>
+        <v>414171</v>
       </c>
       <c r="D3" t="n">
-        <v>45</v>
+        <v>85</v>
       </c>
       <c r="E3" t="n">
-        <v>0.0018</v>
+        <v>0.0205</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily follower scan: 2026-10-24
</commit_message>
<xml_diff>
--- a/daily_report.xlsx
+++ b/daily_report.xlsx
@@ -450,16 +450,16 @@
         </is>
       </c>
       <c r="B2" t="n">
+        <v>2497191</v>
+      </c>
+      <c r="C2" t="n">
         <v>2497091</v>
       </c>
-      <c r="C2" t="n">
-        <v>2496926</v>
-      </c>
       <c r="D2" t="n">
-        <v>165</v>
+        <v>100</v>
       </c>
       <c r="E2" t="n">
-        <v>0.0066</v>
+        <v>0.004</v>
       </c>
     </row>
     <row r="3">
@@ -469,16 +469,16 @@
         </is>
       </c>
       <c r="B3" t="n">
+        <v>414351</v>
+      </c>
+      <c r="C3" t="n">
         <v>414256</v>
       </c>
-      <c r="C3" t="n">
-        <v>414171</v>
-      </c>
       <c r="D3" t="n">
-        <v>85</v>
+        <v>95</v>
       </c>
       <c r="E3" t="n">
-        <v>0.0205</v>
+        <v>0.0229</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily follower scan: 2026-10-25
</commit_message>
<xml_diff>
--- a/daily_report.xlsx
+++ b/daily_report.xlsx
@@ -450,16 +450,16 @@
         </is>
       </c>
       <c r="B2" t="n">
+        <v>2497305</v>
+      </c>
+      <c r="C2" t="n">
         <v>2497191</v>
       </c>
-      <c r="C2" t="n">
-        <v>2497091</v>
-      </c>
       <c r="D2" t="n">
-        <v>100</v>
+        <v>114</v>
       </c>
       <c r="E2" t="n">
-        <v>0.004</v>
+        <v>0.0046</v>
       </c>
     </row>
     <row r="3">
@@ -469,16 +469,16 @@
         </is>
       </c>
       <c r="B3" t="n">
+        <v>414443</v>
+      </c>
+      <c r="C3" t="n">
         <v>414351</v>
       </c>
-      <c r="C3" t="n">
-        <v>414256</v>
-      </c>
       <c r="D3" t="n">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="E3" t="n">
-        <v>0.0229</v>
+        <v>0.0222</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily follower scan: 2026-10-26
</commit_message>
<xml_diff>
--- a/daily_report.xlsx
+++ b/daily_report.xlsx
@@ -446,39 +446,39 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>telkomsel</t>
+          <t>myxl</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>2497305</v>
+        <v>414591</v>
       </c>
       <c r="C2" t="n">
-        <v>2497191</v>
+        <v>414443</v>
       </c>
       <c r="D2" t="n">
-        <v>114</v>
+        <v>148</v>
       </c>
       <c r="E2" t="n">
-        <v>0.0046</v>
+        <v>0.0357</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>myxl</t>
+          <t>telkomsel</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>414443</v>
+        <v>2497403</v>
       </c>
       <c r="C3" t="n">
-        <v>414351</v>
+        <v>2497305</v>
       </c>
       <c r="D3" t="n">
-        <v>92</v>
+        <v>98</v>
       </c>
       <c r="E3" t="n">
-        <v>0.0222</v>
+        <v>0.0039</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily follower scan: 2026-10-27
</commit_message>
<xml_diff>
--- a/daily_report.xlsx
+++ b/daily_report.xlsx
@@ -450,16 +450,16 @@
         </is>
       </c>
       <c r="B2" t="n">
+        <v>414695</v>
+      </c>
+      <c r="C2" t="n">
         <v>414591</v>
       </c>
-      <c r="C2" t="n">
-        <v>414443</v>
-      </c>
       <c r="D2" t="n">
-        <v>148</v>
+        <v>104</v>
       </c>
       <c r="E2" t="n">
-        <v>0.0357</v>
+        <v>0.0251</v>
       </c>
     </row>
     <row r="3">
@@ -469,13 +469,13 @@
         </is>
       </c>
       <c r="B3" t="n">
+        <v>2497500</v>
+      </c>
+      <c r="C3" t="n">
         <v>2497403</v>
       </c>
-      <c r="C3" t="n">
-        <v>2497305</v>
-      </c>
       <c r="D3" t="n">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="E3" t="n">
         <v>0.0039</v>

</xml_diff>

<commit_message>
Daily follower scan: 2026-10-28
</commit_message>
<xml_diff>
--- a/daily_report.xlsx
+++ b/daily_report.xlsx
@@ -450,16 +450,16 @@
         </is>
       </c>
       <c r="B2" t="n">
+        <v>414846</v>
+      </c>
+      <c r="C2" t="n">
         <v>414695</v>
       </c>
-      <c r="C2" t="n">
-        <v>414591</v>
-      </c>
       <c r="D2" t="n">
-        <v>104</v>
+        <v>151</v>
       </c>
       <c r="E2" t="n">
-        <v>0.0251</v>
+        <v>0.0364</v>
       </c>
     </row>
     <row r="3">
@@ -469,16 +469,16 @@
         </is>
       </c>
       <c r="B3" t="n">
+        <v>2497471</v>
+      </c>
+      <c r="C3" t="n">
         <v>2497500</v>
       </c>
-      <c r="C3" t="n">
-        <v>2497403</v>
-      </c>
       <c r="D3" t="n">
-        <v>97</v>
+        <v>-29</v>
       </c>
       <c r="E3" t="n">
-        <v>0.0039</v>
+        <v>-0.0012</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily follower scan: 2026-10-29
</commit_message>
<xml_diff>
--- a/daily_report.xlsx
+++ b/daily_report.xlsx
@@ -450,16 +450,16 @@
         </is>
       </c>
       <c r="B2" t="n">
+        <v>414988</v>
+      </c>
+      <c r="C2" t="n">
         <v>414846</v>
       </c>
-      <c r="C2" t="n">
-        <v>414695</v>
-      </c>
       <c r="D2" t="n">
-        <v>151</v>
+        <v>142</v>
       </c>
       <c r="E2" t="n">
-        <v>0.0364</v>
+        <v>0.0342</v>
       </c>
     </row>
     <row r="3">
@@ -469,16 +469,16 @@
         </is>
       </c>
       <c r="B3" t="n">
+        <v>2497480</v>
+      </c>
+      <c r="C3" t="n">
         <v>2497471</v>
       </c>
-      <c r="C3" t="n">
-        <v>2497500</v>
-      </c>
       <c r="D3" t="n">
-        <v>-29</v>
+        <v>9</v>
       </c>
       <c r="E3" t="n">
-        <v>-0.0012</v>
+        <v>0.0004</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily follower scan: 2026-10-30
</commit_message>
<xml_diff>
--- a/daily_report.xlsx
+++ b/daily_report.xlsx
@@ -450,16 +450,16 @@
         </is>
       </c>
       <c r="B2" t="n">
+        <v>415190</v>
+      </c>
+      <c r="C2" t="n">
         <v>414988</v>
       </c>
-      <c r="C2" t="n">
-        <v>414846</v>
-      </c>
       <c r="D2" t="n">
-        <v>142</v>
+        <v>202</v>
       </c>
       <c r="E2" t="n">
-        <v>0.0342</v>
+        <v>0.0487</v>
       </c>
     </row>
     <row r="3">
@@ -469,16 +469,16 @@
         </is>
       </c>
       <c r="B3" t="n">
+        <v>2497504</v>
+      </c>
+      <c r="C3" t="n">
         <v>2497480</v>
       </c>
-      <c r="C3" t="n">
-        <v>2497471</v>
-      </c>
       <c r="D3" t="n">
-        <v>9</v>
+        <v>24</v>
       </c>
       <c r="E3" t="n">
-        <v>0.0004</v>
+        <v>0.001</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Daily follower scan: 2026-10-31
</commit_message>
<xml_diff>
--- a/daily_report.xlsx
+++ b/daily_report.xlsx
@@ -450,16 +450,16 @@
         </is>
       </c>
       <c r="B2" t="n">
+        <v>415354</v>
+      </c>
+      <c r="C2" t="n">
         <v>415190</v>
       </c>
-      <c r="C2" t="n">
-        <v>414988</v>
-      </c>
       <c r="D2" t="n">
-        <v>202</v>
+        <v>164</v>
       </c>
       <c r="E2" t="n">
-        <v>0.0487</v>
+        <v>0.0395</v>
       </c>
     </row>
     <row r="3">
@@ -469,16 +469,16 @@
         </is>
       </c>
       <c r="B3" t="n">
+        <v>2497569</v>
+      </c>
+      <c r="C3" t="n">
         <v>2497504</v>
       </c>
-      <c r="C3" t="n">
-        <v>2497480</v>
-      </c>
       <c r="D3" t="n">
-        <v>24</v>
+        <v>65</v>
       </c>
       <c r="E3" t="n">
-        <v>0.001</v>
+        <v>0.0026</v>
       </c>
     </row>
   </sheetData>

</xml_diff>